<commit_message>
Aktulizacja Opisu kolumny w finalnej tabeli
</commit_message>
<xml_diff>
--- a/Docs/Tabela_z_nazwami_kolumn_i_komentarzami.xlsx
+++ b/Docs/Tabela_z_nazwami_kolumn_i_komentarzami.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kacpe\OneDrive\Pulpit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studia\IPZ-Pewniaczki\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE3875CF-07BC-4594-BDAC-2B5AF2F5CD00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329D992A-9261-47C9-ABBD-B6290A415F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5748" yWindow="360" windowWidth="17280" windowHeight="8880" xr2:uid="{AA918570-661E-45F6-89F6-738A95499EEA}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{AA918570-661E-45F6-89F6-738A95499EEA}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="119">
   <si>
     <t>Nazwa Kolumny</t>
   </si>
@@ -427,6 +427,54 @@
   </si>
   <si>
     <t>Wzór matematyczny</t>
+  </si>
+  <si>
+    <t>FTHG</t>
+  </si>
+  <si>
+    <t>Ilość zdobytych goli na koniec meczu przez gospodarzy</t>
+  </si>
+  <si>
+    <t>FTAG</t>
+  </si>
+  <si>
+    <t>Ilość zdobytych goli na koniec meczu przez gości</t>
+  </si>
+  <si>
+    <t>HomeMatchday</t>
+  </si>
+  <si>
+    <t>Numer kolejki gospodarzy</t>
+  </si>
+  <si>
+    <t>AwayMatchday</t>
+  </si>
+  <si>
+    <t>Numer kolejki gości</t>
+  </si>
+  <si>
+    <t>isSuprise_H</t>
+  </si>
+  <si>
+    <t>Czy mecz zakończył się niespodzianką gospodarzy</t>
+  </si>
+  <si>
+    <t>Czy mecz zakończył się niespodzianką gości</t>
+  </si>
+  <si>
+    <t>Czy mecz zakończył się niespodzianką remis</t>
+  </si>
+  <si>
+    <t>isSuprise_D</t>
+  </si>
+  <si>
+    <t>isSuprise_A</t>
+  </si>
+  <si>
+    <t>isSuprise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czy mecz zakończył się jaką kolwiek niespodzianką </t>
   </si>
 </sst>
 </file>
@@ -513,29 +561,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="45" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="45" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -965,7 +1013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA06EDAE-231A-4D42-AFF7-DB4624B8F69F}">
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.109375" customWidth="1"/>
@@ -975,661 +1023,719 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="8" t="s">
+      <c r="A15" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="8" t="s">
+      <c r="A16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
+      <c r="A23" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
+      <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
+      <c r="A26" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
+      <c r="A27" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="8" t="s">
+      <c r="B28" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D28" s="5"/>
-      <c r="E28" s="1" t="e" vm="1">
+      <c r="D28" s="1"/>
+      <c r="E28" s="3" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="5"/>
-      <c r="E29" s="1" t="e" vm="2">
+      <c r="D29" s="1"/>
+      <c r="E29" s="3" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="1" t="e" vm="3">
+      <c r="D32" s="1"/>
+      <c r="E32" s="3" t="e" vm="3">
         <v>#VALUE!</v>
       </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="1" t="e" vm="4">
+      <c r="D35" s="1"/>
+      <c r="E35" s="3" t="e" vm="4">
         <v>#VALUE!</v>
       </c>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="4"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D38" s="5"/>
-      <c r="E38" s="1" t="e" vm="5">
+      <c r="D38" s="1"/>
+      <c r="E38" s="3" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
+      <c r="C39" s="5"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D41" s="5"/>
-      <c r="E41" s="1" t="e" vm="6">
+      <c r="D41" s="1"/>
+      <c r="E41" s="3" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="C42" s="3"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C43" s="3"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D44" s="5"/>
-      <c r="E44" s="1" t="e" vm="7">
+      <c r="D44" s="1"/>
+      <c r="E44" s="3" t="e" vm="7">
         <v>#VALUE!</v>
       </c>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C45" s="6"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C46" s="6"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>118</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="C7:C24"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="E38:G40"/>
-    <mergeCell ref="C41:C43"/>
-    <mergeCell ref="E41:G43"/>
     <mergeCell ref="C44:C46"/>
     <mergeCell ref="E44:G46"/>
     <mergeCell ref="C29:C31"/>
@@ -1638,12 +1744,35 @@
     <mergeCell ref="E29:G31"/>
     <mergeCell ref="E32:G34"/>
     <mergeCell ref="E35:G37"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="C7:C24"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="E38:G40"/>
+    <mergeCell ref="C41:C43"/>
+    <mergeCell ref="E41:G43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="06e0fab9-d3c7-4228-8951-a381beafabee" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100898C99BFA6707C449FB5DEFD6C6B88D2" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="4233cc6462d02d07e0ae1fe028f05d54">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="06e0fab9-d3c7-4228-8951-a381beafabee" xmlns:ns4="4d8e724f-ed6c-4b7c-86a4-236d8fc22848" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bc2c63a7dad31bfee6583dfabf5fe5b2" ns3:_="" ns4:_="">
     <xsd:import namespace="06e0fab9-d3c7-4228-8951-a381beafabee"/>
@@ -1864,24 +1993,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{095922AC-C00C-4C3C-BB2B-E0AD90BB0401}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="06e0fab9-d3c7-4228-8951-a381beafabee"/>
+    <ds:schemaRef ds:uri="4d8e724f-ed6c-4b7c-86a4-236d8fc22848"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="06e0fab9-d3c7-4228-8951-a381beafabee" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FCC0122-E133-43C9-9977-532E7FF3F527}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A417F2B-CE74-45A8-BAE5-74E6674E54B9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1898,29 +2035,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9FCC0122-E133-43C9-9977-532E7FF3F527}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{095922AC-C00C-4C3C-BB2B-E0AD90BB0401}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="06e0fab9-d3c7-4228-8951-a381beafabee"/>
-    <ds:schemaRef ds:uri="4d8e724f-ed6c-4b7c-86a4-236d8fc22848"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>